<commit_message>
n8n board refresh 2026-08-02T17:38:46Z
</commit_message>
<xml_diff>
--- a/app/reports/DFNS_research.xlsx
+++ b/app/reports/DFNS_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-28 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-02 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>24.7392</v>
+        <v>27.68</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04595999717712403</v>
+        <v>0.04744999885559082</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>916173.6838701332</v>
+        <v>1010495.014450867</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>24.7392</v>
+        <v>27.68</v>
       </c>
     </row>
     <row r="38">
@@ -1493,14 +1493,14 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>22665404</v>
+        <v>27970502</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
-        <v>-6.23</v>
+        <v>-6.45</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>54.21</v>
+        <v>56.13</v>
       </c>
     </row>
     <row r="6">
@@ -1595,14 +1595,14 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>21257186</v>
+        <v>21953710</v>
       </c>
       <c r="D11" s="33" t="n"/>
       <c r="E11" s="33" t="n">
-        <v>-0.505</v>
+        <v>-0.49</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>20.32</v>
+        <v>19.742</v>
       </c>
     </row>
     <row r="12">
@@ -1633,14 +1633,14 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>48246416</v>
+        <v>46874980</v>
       </c>
       <c r="D13" s="33" t="n"/>
       <c r="E13" s="33" t="n">
-        <v>-0.546</v>
+        <v>-0.537</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>4.359</v>
+        <v>4.283</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-05T17:42:59Z
</commit_message>
<xml_diff>
--- a/app/reports/DFNS_research.xlsx
+++ b/app/reports/DFNS_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-04 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-05 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>47.5101</v>
+        <v>44.7301</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.0463100004196167</v>
+        <v>0.04620999813079834</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>1010495.031582758</v>
+        <v>1010494.946356033</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>47.5101</v>
+        <v>44.7301</v>
       </c>
     </row>
     <row r="38">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>48008720</v>
+        <v>45199540</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>21639246</v>
+        <v>21615734</v>
       </c>
       <c r="D11" s="33" t="n"/>
       <c r="E11" s="33" t="n">
@@ -1633,14 +1633,14 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>46417832</v>
+        <v>45723676</v>
       </c>
       <c r="D13" s="33" t="n"/>
       <c r="E13" s="33" t="n">
-        <v>-0.534</v>
+        <v>-0.532</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>4.261</v>
+        <v>4.242</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-06T17:43:11Z
</commit_message>
<xml_diff>
--- a/app/reports/DFNS_research.xlsx
+++ b/app/reports/DFNS_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-05 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-06 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>44.7301</v>
+        <v>43.44</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04620999813079834</v>
+        <v>0.04668000221252441</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>1010494.946356033</v>
+        <v>1010494.935543278</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>44.7301</v>
+        <v>43.44</v>
       </c>
     </row>
     <row r="38">
@@ -1493,14 +1493,14 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>45199540</v>
+        <v>43895900</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
-        <v>-6.96</v>
+        <v>-6.73</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>60.6</v>
+        <v>58.54</v>
       </c>
     </row>
     <row r="6">
@@ -1595,14 +1595,14 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>21615734</v>
+        <v>19593760</v>
       </c>
       <c r="D11" s="33" t="n"/>
       <c r="E11" s="33" t="n">
-        <v>-0.472</v>
+        <v>-0.479</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>18.988</v>
+        <v>19.266</v>
       </c>
     </row>
     <row r="12">
@@ -1633,14 +1633,14 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>45723676</v>
+        <v>47835688</v>
       </c>
       <c r="D13" s="33" t="n"/>
       <c r="E13" s="33" t="n">
-        <v>-0.532</v>
+        <v>-0.533</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>4.242</v>
+        <v>4.253</v>
       </c>
     </row>
     <row r="15">

</xml_diff>